<commit_message>
added info of transporation to hotel etc.
</commit_message>
<xml_diff>
--- a/comparing hotels.xlsx
+++ b/comparing hotels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\galce\OneDrive\שולחן העבודה\FOLDERS\projects\Fine-Settimana-A-Milano\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57FE40E3-8CD8-4122-8E2D-1FAFEABCFE6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE57748-5EDA-4145-9E35-183521081B94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14303" yWindow="-23" windowWidth="21795" windowHeight="12976" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -134,7 +134,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -515,14 +515,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I24"/>
-  <sheetFormatPr defaultColWidth="16.25" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="16.25" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="8" width="16.25" style="3"/>
     <col min="9" max="9" width="16.25" style="8"/>
     <col min="10" max="16384" width="16.25" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="72" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" ht="72">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -551,7 +551,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="90" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="90">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -580,7 +580,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="55.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="55.5" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>13</v>
       </c>
@@ -609,7 +609,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="90" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" ht="90">
       <c r="A4" s="4" t="s">
         <v>19</v>
       </c>
@@ -638,7 +638,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="72" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="72">
       <c r="A5" s="4" t="s">
         <v>23</v>
       </c>
@@ -667,7 +667,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="36" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" ht="36">
       <c r="A6" s="4" t="s">
         <v>25</v>
       </c>
@@ -696,7 +696,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="18" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" ht="18">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -707,7 +707,7 @@
       <c r="H7" s="5"/>
       <c r="I7" s="10"/>
     </row>
-    <row r="8" spans="1:9" ht="18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" ht="18">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -718,7 +718,7 @@
       <c r="H8" s="5"/>
       <c r="I8" s="10"/>
     </row>
-    <row r="9" spans="1:9" ht="18" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" ht="18">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -729,7 +729,7 @@
       <c r="H9" s="5"/>
       <c r="I9" s="10"/>
     </row>
-    <row r="10" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" ht="15">
       <c r="A10" s="7"/>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -740,7 +740,7 @@
       <c r="H10" s="7"/>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" ht="15">
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -751,7 +751,7 @@
       <c r="H11" s="7"/>
       <c r="I11" s="6"/>
     </row>
-    <row r="12" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" ht="15">
       <c r="A12" s="7"/>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -762,7 +762,7 @@
       <c r="H12" s="7"/>
       <c r="I12" s="6"/>
     </row>
-    <row r="13" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" ht="15">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -773,7 +773,7 @@
       <c r="H13" s="7"/>
       <c r="I13" s="6"/>
     </row>
-    <row r="14" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" ht="15">
       <c r="A14" s="7"/>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -784,7 +784,7 @@
       <c r="H14" s="7"/>
       <c r="I14" s="6"/>
     </row>
-    <row r="15" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" ht="15">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -795,7 +795,7 @@
       <c r="H15" s="7"/>
       <c r="I15" s="6"/>
     </row>
-    <row r="16" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" ht="15">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -806,7 +806,7 @@
       <c r="H16" s="7"/>
       <c r="I16" s="6"/>
     </row>
-    <row r="17" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="15">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -817,7 +817,7 @@
       <c r="H17" s="7"/>
       <c r="I17" s="6"/>
     </row>
-    <row r="18" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="15">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -828,7 +828,7 @@
       <c r="H18" s="7"/>
       <c r="I18" s="6"/>
     </row>
-    <row r="19" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="15">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -839,7 +839,7 @@
       <c r="H19" s="7"/>
       <c r="I19" s="6"/>
     </row>
-    <row r="20" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" ht="15">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -850,7 +850,7 @@
       <c r="H20" s="7"/>
       <c r="I20" s="6"/>
     </row>
-    <row r="21" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="15">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -861,7 +861,7 @@
       <c r="H21" s="7"/>
       <c r="I21" s="6"/>
     </row>
-    <row r="22" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" ht="15">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -872,7 +872,7 @@
       <c r="H22" s="7"/>
       <c r="I22" s="6"/>
     </row>
-    <row r="23" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="15">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -883,7 +883,7 @@
       <c r="H23" s="7"/>
       <c r="I23" s="6"/>
     </row>
-    <row r="24" spans="1:9" ht="15" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="15">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>

</xml_diff>